<commit_message>
leitura utilizando o for
</commit_message>
<xml_diff>
--- a/14-automacao_tarefas/files/teste.xlsx
+++ b/14-automacao_tarefas/files/teste.xlsx
@@ -440,7 +440,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>41%</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -470,7 +470,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>